<commit_message>
Correct guidance rows in the new registries and regenerate all PDFs
The DPP-CEON and Standards-GS1 registries were seeded from the DPP-DPPO
template, so their guidance row still carried the DPP-DPPO example
identifier and ontology vocabulary. Corrected to DPP_CEON_0001 and
GS1_0001 respectively, and the GS1 ontology vocabulary now reads
DPP|DPPO|CEON|GS1.

Regenerated all four registry PDFs from the spreadsheets (landscape,
columns fitted to one page wide, header row repeated on every page).
DPP-CEON and Standards-GS1 get a PDF for the first time.

Verified: DPP-DPPO 7 mappings, DPPO-CEON 14, DPP-CEON 2, Standards-GS1 5.
Each PDF matches its spreadsheet on mapping count and identifiers.
</commit_message>
<xml_diff>
--- a/mappings/Standards-GS1/Standards-GS1.xlsx
+++ b/mappings/Standards-GS1/Standards-GS1.xlsx
@@ -550,12 +550,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Stable mapping identifier, e.g., DPP_DPPO_0001</t>
+          <t>Stable mapping identifier, e.g., GS1_0001</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>DPP|DPPO|CEON</t>
+          <t>DPP|DPPO|CEON|GS1</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>DPP|DPPO|CEON</t>
+          <t>DPP|DPPO|CEON|GS1</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">

</xml_diff>